<commit_message>
Support iERP warehouse SQL export format for Display library
- Parse WarehouseName / Sku / ProductName / DisplayQty from display.xlsx
- Aggregate multiple warehouse rows per product into shop tabs
- Update display.sql with user's Stocks/Warehouses/Products query

Co-authored-by: shawnzhang0509-ai <shawnzhang0509-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/display.xlsx
+++ b/display.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Display" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,161 +413,189 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>product_code</t>
+          <t>WarehouseName</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>product_name</t>
+          <t>Sku</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>product_family</t>
+          <t>ProductName</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>stock_details</t>
+          <t>DisplayQty</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Onehunga Shop-Display</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>ORL-2S</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Orlando 2 seater</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Orlando</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Onehunga Shop-Display:1;Westgate display:1</t>
-        </is>
+      <c r="D2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LIB-3S</t>
+          <t>Westgate display</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>liberty</t>
+          <t>ORL-2S</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>liberty</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Onehunga Shop-Display:1;Hamilton Shop Display:2</t>
-        </is>
+          <t>Orlando 2 seater</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NEB-L</t>
+          <t>Onehunga Shop-Display</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>nebula</t>
+          <t>LIB-3S</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nebula</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>CHCH Display:1;CHCH Display Colombo:2</t>
-        </is>
+          <t>liberty</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FS-01</t>
+          <t>Hamilton Shop Display</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>featherstone</t>
+          <t>LIB-3S</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>featherstone</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Onehunga Shop-Display:1</t>
-        </is>
+          <t>liberty</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XMAS-RD</t>
+          <t>CHCH Display</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>xmas round</t>
+          <t>NEB-L</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>xmas</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Westgate display:2;Hamilton Shop Display:1</t>
-        </is>
+          <t>nebula</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Onehunga Shop-Display</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FS-01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>featherstone</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Westgate display</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>XMAS-RD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>xmas round</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Onehunga Shop-Display</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>AUR-3S</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Aurora 3 seater</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Aurora</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Onehunga Shop-Display:1;CHCH Gerald Connelly:1</t>
-        </is>
+      <c r="D9" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>